<commit_message>
valving and diff FF calculations
</commit_message>
<xml_diff>
--- a/docs/diff_map.xlsx
+++ b/docs/diff_map.xlsx
@@ -432,19 +432,19 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.86891310437455982</c:v>
+                  <c:v>0.8689131043745597</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.76634591660498397</c:v>
+                  <c:v>0.7058823529411764</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.6658880094220041</c:v>
+                  <c:v>0.6133504266173363</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.59786370542100298</c:v>
+                  <c:v>0.597863705421003</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.45817040933571068</c:v>
+                  <c:v>0.422021439120708</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -675,19 +675,19 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.80904494997656273</c:v>
+                  <c:v>0.8090449499765627</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.76634591660498397</c:v>
+                  <c:v>0.7058823529411765</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.65557648104589672</c:v>
+                  <c:v>0.6555764810458966</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.62000829376442235</c:v>
+                  <c:v>0.5710905529246325</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.50239835927178755</c:v>
+                  <c:v>0.4627598689735741</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -912,13 +912,13 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.76634591660498397</c:v>
+                  <c:v>0.7058823529411764</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.54267864568626134</c:v>
+                  <c:v>0.5426786456862612</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.41587956415038935</c:v>
+                  <c:v>0.3830672793079491</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1422,21 +1422,12 @@
     </row>
     <row r="3" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="2">
-        <f t="shared" ref="B3:B4" si="0">(1/TAN(46*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(A3-8)*0.0947)*2</f>
-        <v>0.10653932410387595</v>
-      </c>
+      <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="2">
-        <f t="shared" ref="D3:D8" si="1">(1/TAN(72*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(A3-8)*0.0947)*2</f>
-        <v>3.5846667920113581E-2</v>
-      </c>
+      <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2">
-        <f t="shared" ref="G3:G4" si="2">(1/TAN(38*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(F3-8)*0.0947)*2</f>
-        <v>0.14120917623124007</v>
-      </c>
+      <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -1445,21 +1436,16 @@
     </row>
     <row r="4" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="12">
-        <f t="shared" si="0"/>
-        <v>0.10653932410387595</v>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>相对值以各图注明的参考组合为 100%；完整系数与模型等效百分比见 Samples。</t>
+        </is>
       </c>
       <c r="C4" s="12"/>
-      <c r="D4" s="12">
-        <f t="shared" si="1"/>
-        <v>3.5846667920113581E-2</v>
-      </c>
+      <c r="D4" s="12"/>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
-      <c r="G4" s="12">
-        <f t="shared" si="2"/>
-        <v>0.14120917623124007</v>
-      </c>
+      <c r="G4" s="12"/>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
       <c r="J4" s="12"/>
@@ -1499,18 +1485,12 @@
     </row>
     <row r="7" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
-      <c r="B7" s="2">
-        <f t="shared" ref="B7:B8" si="3">(1/TAN(50*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(A7-8)*0.0947)*2</f>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="2">
-        <f t="shared" ref="G7:G8" si="4">(1/TAN(44*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(F7-8)*0.0947)*2</f>
-        <v>0.11424457092023524</v>
-      </c>
+      <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -1519,21 +1499,12 @@
     </row>
     <row r="8" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
-      <c r="B8" s="2">
-        <f t="shared" si="3"/>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="2">
-        <f t="shared" si="1"/>
-        <v>3.5846667920113581E-2</v>
-      </c>
+      <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="2">
-        <f t="shared" si="4"/>
-        <v>0.11424457092023524</v>
-      </c>
+      <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -1570,18 +1541,12 @@
     </row>
     <row r="11" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
-      <c r="B11" s="2">
-        <f t="shared" ref="B11:B12" si="5">(1/TAN(60*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(A11-8)*0.0947)*2</f>
-        <v>6.3695995081792453E-2</v>
-      </c>
+      <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
-      <c r="G11" s="2">
-        <f t="shared" ref="G11:G12" si="6">(1/TAN(50*PI()/180))/(1/TAN(35*PI()/180))*0.325*(1+(F11-8)*0.0947)*2</f>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -1590,18 +1555,12 @@
     </row>
     <row r="12" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
-      <c r="B12" s="2">
-        <f t="shared" si="5"/>
-        <v>6.3695995081792453E-2</v>
-      </c>
+      <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="2">
-        <f t="shared" si="6"/>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -1652,18 +1611,12 @@
     </row>
     <row r="16" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
-      <c r="B16" s="2">
-        <f t="shared" ref="B16:B17" si="7">B3</f>
-        <v>0.10653932410387595</v>
-      </c>
+      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="2">
-        <f t="shared" ref="G16:G17" si="8">G3</f>
-        <v>0.14120917623124007</v>
-      </c>
+      <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -1672,18 +1625,12 @@
     </row>
     <row r="17" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
-      <c r="B17" s="2">
-        <f t="shared" si="7"/>
-        <v>0.10653932410387595</v>
-      </c>
+      <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="2">
-        <f t="shared" si="8"/>
-        <v>0.14120917623124007</v>
-      </c>
+      <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -1692,18 +1639,12 @@
     </row>
     <row r="18" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
-      <c r="B18" s="2">
-        <f t="shared" ref="B18:B19" si="9">B7</f>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="2">
-        <f t="shared" ref="G18:G19" si="10">G7</f>
-        <v>0.11424457092023524</v>
-      </c>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -1712,18 +1653,12 @@
     </row>
     <row r="19" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="2">
-        <f t="shared" si="9"/>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="2">
-        <f t="shared" si="10"/>
-        <v>0.11424457092023524</v>
-      </c>
+      <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1732,18 +1667,12 @@
     </row>
     <row r="20" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
-      <c r="B20" s="2">
-        <f t="shared" ref="B20:B21" si="11">B11</f>
-        <v>6.3695995081792453E-2</v>
-      </c>
+      <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="2">
-        <f t="shared" ref="G20:G21" si="12">G11</f>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -1752,18 +1681,15 @@
     </row>
     <row r="21" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
-      <c r="B21" s="13">
-        <f t="shared" si="11"/>
-        <v>6.3695995081792453E-2</v>
+      <c r="B21" s="13" t="str">
+        <f>"Rear power："&amp;Samples!E12&amp;" = 100%"</f>
+        <v>Rear power：38° / 6+6 = 100%</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
       <c r="F21" s="13"/>
-      <c r="G21" s="13">
-        <f t="shared" si="12"/>
-        <v>9.2573414845066218E-2</v>
-      </c>
+      <c r="G21" s="13"/>
       <c r="H21" s="13"/>
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
@@ -1772,18 +1698,12 @@
     </row>
     <row r="22" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
-      <c r="B22" s="2">
-        <f t="shared" ref="B22:B23" si="13">D3</f>
-        <v>3.5846667920113581E-2</v>
-      </c>
+      <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="2">
-        <f t="shared" ref="G22:G23" si="14">H3</f>
-        <v>0</v>
-      </c>
+      <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -1792,18 +1712,12 @@
     </row>
     <row r="23" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
-      <c r="B23" s="2">
-        <f t="shared" si="13"/>
-        <v>3.5846667920113581E-2</v>
-      </c>
+      <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="2">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
+      <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -1812,10 +1726,7 @@
     </row>
     <row r="24" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
-      <c r="B24" s="2">
-        <f t="shared" ref="B24:B25" si="15">C3</f>
-        <v>0</v>
-      </c>
+      <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1829,10 +1740,7 @@
     </row>
     <row r="25" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
-      <c r="B25" s="2">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -2409,7 +2317,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>11</v>
@@ -2435,20 +2343,22 @@
         <v>13</v>
       </c>
       <c r="C9" s="5">
-        <v>0.32500000000000001</v>
+        <v>0.20189</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="2" t="s">
-        <v>15</v>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>锚点 / 原 Q6</t>
+        </is>
       </c>
       <c r="G9" s="4">
         <v>35</v>
       </c>
       <c r="H9" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -2461,7 +2371,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="5">
-        <v>9.4700000000000006E-2</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>14</v>
@@ -2789,8 +2699,10 @@
     </row>
     <row r="28" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="B28" s="16" t="s">
-        <v>32</v>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>模型等效百分比 = c × 换算倍数；35°、4+4 的 c = 0.20189，对应 40.378%。</t>
+        </is>
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
@@ -2869,8 +2781,10 @@
     </row>
     <row r="33" spans="1:12" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
-      <c r="B33" s="12" t="s">
-        <v>37</v>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>FF 折中标定：保留 4+4；每侧增加一面，锚点系数增加 5/24。</t>
+        </is>
       </c>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
@@ -3060,14 +2974,14 @@
       </c>
       <c r="F6" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C6*PI()/180)*Parameters!$C$9*(1+(D6-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.17813691443605995</v>
+        <v>0.19339553738080512</v>
       </c>
       <c r="G6" s="8">
         <f>F6*Parameters!$C$11</f>
-        <v>0.35627382887211989</v>
+        <v>0.38679107476161023</v>
       </c>
       <c r="H6" s="8">
-        <f t="shared" ref="H6:H11" si="1">G6/$G$6</f>
+        <f>G6/$G$6</f>
         <v>1</v>
       </c>
       <c r="I6" s="2"/>
@@ -3092,15 +3006,15 @@
       </c>
       <c r="F7" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C7*PI()/180)*Parameters!$C$9*(1+(D7-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.1547854993263422</v>
+        <v>0.16804391675774158</v>
       </c>
       <c r="G7" s="8">
         <f>F7*Parameters!$C$11</f>
-        <v>0.30957099865268439</v>
+        <v>0.33608783351548316</v>
       </c>
       <c r="H7" s="8">
-        <f t="shared" si="1"/>
-        <v>0.86891310437455982</v>
+        <f>G7/$G$6</f>
+        <v>0.8689131043745597</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -3128,11 +3042,11 @@
       </c>
       <c r="G8" s="8">
         <f>F8*Parameters!$C$11</f>
-        <v>0.27302899394937191</v>
+        <v>0.2730289939493719</v>
       </c>
       <c r="H8" s="8">
-        <f t="shared" si="1"/>
-        <v>0.76634591660498397</v>
+        <f>G8/$G$6</f>
+        <v>0.7058823529411764</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -3163,8 +3077,8 @@
         <v>0.23723847071681164</v>
       </c>
       <c r="H9" s="8">
-        <f t="shared" si="1"/>
-        <v>0.6658880094220041</v>
+        <f>G9/$G$6</f>
+        <v>0.6133504266173363</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -3188,15 +3102,15 @@
       </c>
       <c r="F10" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C10*PI()/180)*Parameters!$C$9*(1+(D10-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.10650159573700696</v>
+        <v>0.11562417259037425</v>
       </c>
       <c r="G10" s="8">
         <f>F10*Parameters!$C$11</f>
-        <v>0.21300319147401392</v>
+        <v>0.2312483451807485</v>
       </c>
       <c r="H10" s="8">
-        <f t="shared" si="1"/>
-        <v>0.59786370542100298</v>
+        <f>G10/$G$6</f>
+        <v>0.597863705421003</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -3220,15 +3134,15 @@
       </c>
       <c r="F11" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C11*PI()/180)*Parameters!$C$9*(1+(D11-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>8.1617063004970056E-2</v>
+        <v>0.08161706300497006</v>
       </c>
       <c r="G11" s="8">
         <f>F11*Parameters!$C$11</f>
-        <v>0.16323412600994011</v>
+        <v>0.1632341260099401</v>
       </c>
       <c r="H11" s="8">
-        <f t="shared" si="1"/>
-        <v>0.45817040933571068</v>
+        <f>G11/$G$6</f>
+        <v>0.422021439120708</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -3252,14 +3166,14 @@
       </c>
       <c r="F12" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C12*PI()/180)*Parameters!$C$9*(1+(D12-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.23610593699060067</v>
+        <v>0.25632999599016565</v>
       </c>
       <c r="G12" s="8">
         <f>F12*Parameters!$C$11</f>
-        <v>0.47221187398120135</v>
+        <v>0.5126599919803313</v>
       </c>
       <c r="H12" s="8">
-        <f t="shared" ref="H12:H17" si="2">G12/$G$12</f>
+        <f>G12/$G$12</f>
         <v>1</v>
       </c>
       <c r="I12" s="2"/>
@@ -3284,15 +3198,15 @@
       </c>
       <c r="F13" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C13*PI()/180)*Parameters!$C$9*(1+(D13-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.19102031598173</v>
+        <v>0.2073824887833561</v>
       </c>
       <c r="G13" s="8">
         <f>F13*Parameters!$C$11</f>
-        <v>0.38204063196346</v>
+        <v>0.4147649775667122</v>
       </c>
       <c r="H13" s="8">
-        <f t="shared" si="2"/>
-        <v>0.80904494997656273</v>
+        <f>G13/$G$12</f>
+        <v>0.8090449499765627</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -3320,11 +3234,11 @@
       </c>
       <c r="G14" s="8">
         <f>F14*Parameters!$C$11</f>
-        <v>0.36187764139788092</v>
+        <v>0.3618776413978809</v>
       </c>
       <c r="H14" s="8">
-        <f t="shared" si="2"/>
-        <v>0.76634591660498397</v>
+        <f>G14/$G$12</f>
+        <v>0.7058823529411765</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -3348,15 +3262,15 @@
       </c>
       <c r="F15" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C15*PI()/180)*Parameters!$C$9*(1+(D15-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.1547854993263422</v>
+        <v>0.16804391675774158</v>
       </c>
       <c r="G15" s="8">
         <f>F15*Parameters!$C$11</f>
-        <v>0.30957099865268439</v>
+        <v>0.33608783351548316</v>
       </c>
       <c r="H15" s="8">
-        <f t="shared" si="2"/>
-        <v>0.65557648104589672</v>
+        <f>G15/$G$12</f>
+        <v>0.6555764810458966</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -3384,11 +3298,11 @@
       </c>
       <c r="G16" s="8">
         <f>F16*Parameters!$C$11</f>
-        <v>0.29277527828238509</v>
+        <v>0.2927752782823851</v>
       </c>
       <c r="H16" s="8">
-        <f t="shared" si="2"/>
-        <v>0.62000829376442235</v>
+        <f>G16/$G$12</f>
+        <v>0.5710905529246325</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -3419,8 +3333,8 @@
         <v>0.23723847071681164</v>
       </c>
       <c r="H17" s="8">
-        <f t="shared" si="2"/>
-        <v>0.50239835927178755</v>
+        <f>G17/$G$12</f>
+        <v>0.4627598689735741</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3444,11 +3358,11 @@
       </c>
       <c r="F18" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C18*PI()/180)*Parameters!$C$9*(1+(D18-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>5.99366935149424E-2</v>
+        <v>0.06507067380080576</v>
       </c>
       <c r="G18" s="8">
         <f>F18*Parameters!$C$11</f>
-        <v>0.1198733870298848</v>
+        <v>0.13014134760161153</v>
       </c>
       <c r="H18" s="8">
         <f>G18/$G$18</f>
@@ -3476,15 +3390,15 @@
       </c>
       <c r="F19" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C19*PI()/180)*Parameters!$C$9*(1+(D19-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>4.5932240329980535E-2</v>
+        <v>0.045932240329980535</v>
       </c>
       <c r="G19" s="8">
         <f>F19*Parameters!$C$11</f>
-        <v>9.186448065996107E-2</v>
+        <v>0.09186448065996107</v>
       </c>
       <c r="H19" s="8">
         <f>G19/$G$18</f>
-        <v>0.76634591660498397</v>
+        <v>0.7058823529411764</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -3508,15 +3422,15 @@
       </c>
       <c r="F20" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C20*PI()/180)*Parameters!$C$9*(1+(D20-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>3.2526363663601468E-2</v>
+        <v>0.03531246513211375</v>
       </c>
       <c r="G20" s="8">
         <f>F20*Parameters!$C$11</f>
-        <v>6.5052727327202936E-2</v>
+        <v>0.0706249302642275</v>
       </c>
       <c r="H20" s="8">
         <f>G20/$G$18</f>
-        <v>0.54267864568626134</v>
+        <v>0.5426786456862612</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -3540,15 +3454,15 @@
       </c>
       <c r="F21" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C21*PI()/180)*Parameters!$C$9*(1+(D21-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>2.4926445975609713E-2</v>
+        <v>0.024926445975609706</v>
       </c>
       <c r="G21" s="8">
         <f>F21*Parameters!$C$11</f>
-        <v>4.9852891951219426E-2</v>
+        <v>0.04985289195121941</v>
       </c>
       <c r="H21" s="8">
         <f>G21/$G$18</f>
-        <v>0.41587956415038935</v>
+        <v>0.3830672793079491</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -3572,11 +3486,11 @@
       </c>
       <c r="F22" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C22*PI()/180)*Parameters!$C$9*(1+(D22-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.16847212730962527</v>
+        <v>0.16847212730962524</v>
       </c>
       <c r="G22" s="8">
         <f>F22*Parameters!$C$11</f>
-        <v>0.33694425461925054</v>
+        <v>0.3369442546192505</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="2"/>
@@ -3593,7 +3507,7 @@
       </c>
       <c r="D23" s="9">
         <f>Parameters!H9</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E23" s="2" t="str">
         <f t="shared" si="0"/>
@@ -3601,11 +3515,11 @@
       </c>
       <c r="F23" s="7">
         <f>TAN(Parameters!$C$7*PI()/180)/TAN(C23*PI()/180)*Parameters!$C$9*(1+(D23-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.32500000000000001</v>
+        <v>0.20189</v>
       </c>
       <c r="G23" s="8">
         <f>F23*Parameters!$C$11</f>
-        <v>0.65</v>
+        <v>0.40378</v>
       </c>
       <c r="H23" s="8"/>
       <c r="I23" s="2"/>

</xml_diff>

<commit_message>
Refine differential ramp calibration and rally setups
</commit_message>
<xml_diff>
--- a/docs/diff_map.xlsx
+++ b/docs/diff_map.xlsx
@@ -615,7 +615,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -697,6 +697,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -765,13 +768,13 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>45° / 6+6</c:v>
+                  <c:v>46° / 6+6</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>50° / 6+6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45° / 4+4</c:v>
+                  <c:v>46° / 4+4</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>50° / 4+4</c:v>
@@ -795,19 +798,19 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.83909963117727993</c:v>
+                  <c:v>0.8646842979195788</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.70466321243523333</c:v>
+                  <c:v>0.6666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.59128264165860145</c:v>
+                  <c:v>0.5764561986130526</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.53170943166147877</c:v>
+                  <c:v>0.5241827435579796</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.37467607619668974</c:v>
+                  <c:v>0.34945516237198637</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1009,22 +1012,22 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>38° / 6+6</c:v>
+                  <c:v>40° / 6+6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45° / 6+6</c:v>
+                  <c:v>46° / 6+6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>38° / 4+4</c:v>
+                  <c:v>40° / 4+4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>50° / 6+6</c:v>
+                  <c:v>54° / 6+6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45° / 4+4</c:v>
+                  <c:v>46° / 4+4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50° / 4+4</c:v>
+                  <c:v>54° / 4+4</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1039,19 +1042,19 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.78128562650671751</c:v>
+                  <c:v>0.8097840331950072</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.70466321243523333</c:v>
+                  <c:v>0.6666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.65557648104589672</c:v>
+                  <c:v>0.6008606190275605</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.55054323940369743</c:v>
+                  <c:v>0.5398560221300048</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.46196062913078734</c:v>
+                  <c:v>0.4005737460183737</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1259,10 +1262,10 @@
                   <c:v>70° / 4+4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>85° / 6+6</c:v>
+                  <c:v>80° / 6+6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>85° / 4+4</c:v>
+                  <c:v>80° / 4+4</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1277,13 +1280,13 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.70466321243523322</c:v>
+                  <c:v>0.6666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.24037312749573927</c:v>
+                  <c:v>0.3265121373650463</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.16938210020425151</c:v>
+                  <c:v>0.21767475824336424</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1808,7 +1811,7 @@
       <c r="A5" s="2"/>
       <c r="B5" s="25" t="str">
         <f>"Front power："&amp;Samples!E6&amp;" = 100%"</f>
-        <v>Front power：45° / 6+6 = 100%</v>
+        <v>Front power：46° / 6+6 = 100%</v>
       </c>
       <c r="C5" s="25"/>
       <c r="D5" s="25"/>
@@ -2035,7 +2038,7 @@
       <c r="A21" s="2"/>
       <c r="B21" s="25" t="str">
         <f>"Rear power："&amp;Samples!E12&amp;" = 100%"</f>
-        <v>Rear power：38° / 6+6 = 100%</v>
+        <v>Rear power：40° / 6+6 = 100%</v>
       </c>
       <c r="C21" s="25"/>
       <c r="D21" s="25"/>
@@ -2626,11 +2629,13 @@
     </row>
     <row r="7" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
-      <c r="B7" s="4" t="s">
-        <v>3</v>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Ramp 角度补偿</t>
+        </is>
       </c>
       <c r="C7" s="5">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>4</v>
@@ -2662,8 +2667,10 @@
         <v>9</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="4" t="s">
-        <v>10</v>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>校核 1</t>
+        </is>
       </c>
       <c r="G8" s="5">
         <v>40</v>
@@ -2678,18 +2685,22 @@
     </row>
     <row r="9" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
-      <c r="B9" s="4" t="s">
-        <v>11</v>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>基础游戏系数</t>
+        </is>
       </c>
       <c r="C9" s="10">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="8" t="s">
-        <v>29</v>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>校核 2</t>
+        </is>
       </c>
       <c r="G9" s="5">
         <v>35</v>
@@ -2704,15 +2715,9 @@
     </row>
     <row r="10" spans="1:12" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="10">
-        <v>0.114</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -2816,7 +2821,7 @@
         <v>19</v>
       </c>
       <c r="C16" s="5">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -2880,7 +2885,7 @@
         <v>20</v>
       </c>
       <c r="C19" s="5">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -2892,7 +2897,7 @@
         <v>20</v>
       </c>
       <c r="C20" s="5">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -2904,7 +2909,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="5">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -2928,7 +2933,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="5">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -3131,26 +3136,26 @@
       </c>
       <c r="C6" s="15">
         <f>Parameters!C16</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D6" s="15">
         <f>Parameters!G17</f>
         <v>6</v>
       </c>
       <c r="E6" s="11" t="str">
-        <f t="shared" ref="E6:E23" si="0">C6&amp;"° / "&amp;D6&amp;"+"&amp;D6</f>
-        <v>45° / 6+6</v>
+        <f>C6&amp;"° / "&amp;D6&amp;"+"&amp;D6</f>
+        <v>46° / 6+6</v>
       </c>
       <c r="F6" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C6*PI()/180)*Parameters!$C$9*(1+(D6-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.20000728121422151</v>
+        <f>Parameters!$C$9*(D6/Parameters!$C$8)/TAN((C6+Parameters!$C$7)*PI()/180)</f>
+        <v>0.2125683087136894</v>
       </c>
       <c r="G6" s="17">
         <f>F6*Parameters!$C$11</f>
-        <v>0.40001456242844302</v>
+        <v>0.4251366174273788</v>
       </c>
       <c r="H6" s="17">
-        <f t="shared" ref="H6:H11" si="1">G6/$G$6</f>
+        <f>G6/$G$6</f>
         <v>1</v>
       </c>
       <c r="I6" s="2"/>
@@ -3170,20 +3175,20 @@
         <v>6</v>
       </c>
       <c r="E7" s="12" t="str">
-        <f t="shared" si="0"/>
+        <f>C7&amp;"° / "&amp;D7&amp;"+"&amp;D7</f>
         <v>50° / 6+6</v>
       </c>
       <c r="F7" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C7*PI()/180)*Parameters!$C$9*(1+(D7-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.16782603589962378</v>
+        <f>Parameters!$C$9*(D7/Parameters!$C$8)/TAN((C7+Parameters!$C$7)*PI()/180)</f>
+        <v>0.1838044787800488</v>
       </c>
       <c r="G7" s="20">
         <f>F7*Parameters!$C$11</f>
-        <v>0.33565207179924755</v>
+        <v>0.3676089575600976</v>
       </c>
       <c r="H7" s="20">
-        <f t="shared" si="1"/>
-        <v>0.83909963117727993</v>
+        <f>G7/$G$6</f>
+        <v>0.8646842979195788</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -3195,27 +3200,27 @@
       </c>
       <c r="C8" s="15">
         <f>Parameters!C16</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="15">
         <f>Parameters!G16</f>
         <v>4</v>
       </c>
       <c r="E8" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>45° / 4+4</v>
+        <f>C8&amp;"° / "&amp;D8&amp;"+"&amp;D8</f>
+        <v>46° / 4+4</v>
       </c>
       <c r="F8" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C8*PI()/180)*Parameters!$C$9*(1+(D8-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.14093777329085042</v>
+        <f>Parameters!$C$9*(D8/Parameters!$C$8)/TAN((C8+Parameters!$C$7)*PI()/180)</f>
+        <v>0.14171220580912627</v>
       </c>
       <c r="G8" s="17">
         <f>F8*Parameters!$C$11</f>
-        <v>0.28187554658170083</v>
+        <v>0.28342441161825255</v>
       </c>
       <c r="H8" s="17">
-        <f t="shared" si="1"/>
-        <v>0.70466321243523333</v>
+        <f>G8/$G$6</f>
+        <v>0.6666666666666667</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -3234,20 +3239,20 @@
         <v>4</v>
       </c>
       <c r="E9" s="12" t="str">
-        <f t="shared" si="0"/>
+        <f>C9&amp;"° / "&amp;D9&amp;"+"&amp;D9</f>
         <v>50° / 4+4</v>
       </c>
       <c r="F9" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C9*PI()/180)*Parameters!$C$9*(1+(D9-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.11826083358729966</v>
+        <f>Parameters!$C$9*(D9/Parameters!$C$8)/TAN((C9+Parameters!$C$7)*PI()/180)</f>
+        <v>0.12253631918669922</v>
       </c>
       <c r="G9" s="20">
         <f>F9*Parameters!$C$11</f>
-        <v>0.23652166717459933</v>
+        <v>0.24507263837339843</v>
       </c>
       <c r="H9" s="20">
-        <f t="shared" si="1"/>
-        <v>0.59128264165860145</v>
+        <f>G9/$G$6</f>
+        <v>0.5764561986130526</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -3266,20 +3271,20 @@
         <v>6</v>
       </c>
       <c r="E10" s="11" t="str">
-        <f t="shared" si="0"/>
+        <f>C10&amp;"° / "&amp;D10&amp;"+"&amp;D10</f>
         <v>62° / 6+6</v>
       </c>
       <c r="F10" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C10*PI()/180)*Parameters!$C$9*(1+(D10-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.10634575782257129</v>
+        <f>Parameters!$C$9*(D10/Parameters!$C$8)/TAN((C10+Parameters!$C$7)*PI()/180)</f>
+        <v>0.11142463925502127</v>
       </c>
       <c r="G10" s="17">
         <f>F10*Parameters!$C$11</f>
-        <v>0.21269151564514258</v>
+        <v>0.22284927851004255</v>
       </c>
       <c r="H10" s="17">
-        <f t="shared" si="1"/>
-        <v>0.53170943166147877</v>
+        <f>G10/$G$6</f>
+        <v>0.5241827435579796</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -3298,20 +3303,20 @@
         <v>4</v>
       </c>
       <c r="E11" s="12" t="str">
-        <f t="shared" si="0"/>
+        <f>C11&amp;"° / "&amp;D11&amp;"+"&amp;D11</f>
         <v>62° / 4+4</v>
       </c>
       <c r="F11" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C11*PI()/180)*Parameters!$C$9*(1+(D11-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>7.4937943336112409E-2</v>
+        <f>Parameters!$C$9*(D11/Parameters!$C$8)/TAN((C11+Parameters!$C$7)*PI()/180)</f>
+        <v>0.07428309283668086</v>
       </c>
       <c r="G11" s="20">
         <f>F11*Parameters!$C$11</f>
-        <v>0.14987588667222482</v>
+        <v>0.14856618567336172</v>
       </c>
       <c r="H11" s="20">
-        <f t="shared" si="1"/>
-        <v>0.37467607619668974</v>
+        <f>G11/$G$6</f>
+        <v>0.34945516237198637</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -3323,26 +3328,26 @@
       </c>
       <c r="C12" s="15">
         <f>Parameters!C19</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D12" s="15">
         <f>Parameters!G17</f>
         <v>6</v>
       </c>
       <c r="E12" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>38° / 6+6</v>
+        <f>C12&amp;"° / "&amp;D12&amp;"+"&amp;D12</f>
+        <v>40° / 6+6</v>
       </c>
       <c r="F12" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C12*PI()/180)*Parameters!$C$9*(1+(D12-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.25599764596783076</v>
+        <f>Parameters!$C$9*(D12/Parameters!$C$8)/TAN((C12+Parameters!$C$7)*PI()/180)</f>
+        <v>0.2625</v>
       </c>
       <c r="G12" s="17">
         <f>F12*Parameters!$C$11</f>
-        <v>0.51199529193566151</v>
+        <v>0.525</v>
       </c>
       <c r="H12" s="17">
-        <f t="shared" ref="H12:H17" si="2">G12/$G$12</f>
+        <f>G12/$G$12</f>
         <v>1</v>
       </c>
       <c r="I12" s="2"/>
@@ -3355,27 +3360,27 @@
       </c>
       <c r="C13" s="18">
         <f>Parameters!C20</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D13" s="18">
         <f>Parameters!G17</f>
         <v>6</v>
       </c>
       <c r="E13" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>45° / 6+6</v>
+        <f>C13&amp;"° / "&amp;D13&amp;"+"&amp;D13</f>
+        <v>46° / 6+6</v>
       </c>
       <c r="F13" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C13*PI()/180)*Parameters!$C$9*(1+(D13-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.20000728121422151</v>
+        <f>Parameters!$C$9*(D13/Parameters!$C$8)/TAN((C13+Parameters!$C$7)*PI()/180)</f>
+        <v>0.2125683087136894</v>
       </c>
       <c r="G13" s="20">
         <f>F13*Parameters!$C$11</f>
-        <v>0.40001456242844302</v>
+        <v>0.4251366174273788</v>
       </c>
       <c r="H13" s="20">
-        <f t="shared" si="2"/>
-        <v>0.78128562650671751</v>
+        <f>G13/$G$12</f>
+        <v>0.8097840331950072</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -3387,27 +3392,27 @@
       </c>
       <c r="C14" s="15">
         <f>Parameters!C19</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D14" s="15">
         <f>Parameters!G16</f>
         <v>4</v>
       </c>
       <c r="E14" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>38° / 4+4</v>
+        <f>C14&amp;"° / "&amp;D14&amp;"+"&amp;D14</f>
+        <v>40° / 4+4</v>
       </c>
       <c r="F14" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C14*PI()/180)*Parameters!$C$9*(1+(D14-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.18039212358354917</v>
+        <f>Parameters!$C$9*(D14/Parameters!$C$8)/TAN((C14+Parameters!$C$7)*PI()/180)</f>
+        <v>0.17500000000000002</v>
       </c>
       <c r="G14" s="17">
         <f>F14*Parameters!$C$11</f>
-        <v>0.36078424716709834</v>
+        <v>0.35000000000000003</v>
       </c>
       <c r="H14" s="17">
-        <f t="shared" si="2"/>
-        <v>0.70466321243523333</v>
+        <f>G14/$G$12</f>
+        <v>0.6666666666666667</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -3419,27 +3424,27 @@
       </c>
       <c r="C15" s="18">
         <f>Parameters!C21</f>
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D15" s="18">
         <f>Parameters!G17</f>
         <v>6</v>
       </c>
       <c r="E15" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>50° / 6+6</v>
+        <f>C15&amp;"° / "&amp;D15&amp;"+"&amp;D15</f>
+        <v>54° / 6+6</v>
       </c>
       <c r="F15" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C15*PI()/180)*Parameters!$C$9*(1+(D15-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.16782603589962378</v>
+        <f>Parameters!$C$9*(D15/Parameters!$C$8)/TAN((C15+Parameters!$C$7)*PI()/180)</f>
+        <v>0.15772591249473464</v>
       </c>
       <c r="G15" s="20">
         <f>F15*Parameters!$C$11</f>
-        <v>0.33565207179924755</v>
+        <v>0.3154518249894693</v>
       </c>
       <c r="H15" s="20">
-        <f t="shared" si="2"/>
-        <v>0.65557648104589672</v>
+        <f>G15/$G$12</f>
+        <v>0.6008606190275605</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -3451,27 +3456,27 @@
       </c>
       <c r="C16" s="15">
         <f>Parameters!C20</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D16" s="15">
         <f>Parameters!G16</f>
         <v>4</v>
       </c>
       <c r="E16" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>45° / 4+4</v>
+        <f>C16&amp;"° / "&amp;D16&amp;"+"&amp;D16</f>
+        <v>46° / 4+4</v>
       </c>
       <c r="F16" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C16*PI()/180)*Parameters!$C$9*(1+(D16-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.14093777329085042</v>
+        <f>Parameters!$C$9*(D16/Parameters!$C$8)/TAN((C16+Parameters!$C$7)*PI()/180)</f>
+        <v>0.14171220580912627</v>
       </c>
       <c r="G16" s="17">
         <f>F16*Parameters!$C$11</f>
-        <v>0.28187554658170083</v>
+        <v>0.28342441161825255</v>
       </c>
       <c r="H16" s="17">
-        <f t="shared" si="2"/>
-        <v>0.55054323940369743</v>
+        <f>G16/$G$12</f>
+        <v>0.5398560221300048</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -3483,27 +3488,27 @@
       </c>
       <c r="C17" s="18">
         <f>Parameters!C21</f>
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D17" s="18">
         <f>Parameters!G16</f>
         <v>4</v>
       </c>
       <c r="E17" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>50° / 4+4</v>
+        <f>C17&amp;"° / "&amp;D17&amp;"+"&amp;D17</f>
+        <v>54° / 4+4</v>
       </c>
       <c r="F17" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C17*PI()/180)*Parameters!$C$9*(1+(D17-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.11826083358729966</v>
+        <f>Parameters!$C$9*(D17/Parameters!$C$8)/TAN((C17+Parameters!$C$7)*PI()/180)</f>
+        <v>0.1051506083298231</v>
       </c>
       <c r="G17" s="20">
         <f>F17*Parameters!$C$11</f>
-        <v>0.23652166717459933</v>
+        <v>0.2103012166596462</v>
       </c>
       <c r="H17" s="20">
-        <f t="shared" si="2"/>
-        <v>0.46196062913078734</v>
+        <f>G17/$G$12</f>
+        <v>0.4005737460183737</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3522,16 +3527,16 @@
         <v>6</v>
       </c>
       <c r="E18" s="11" t="str">
-        <f t="shared" si="0"/>
+        <f>C18&amp;"° / "&amp;D18&amp;"+"&amp;D18</f>
         <v>70° / 6+6</v>
       </c>
       <c r="F18" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C18*PI()/180)*Parameters!$C$9*(1+(D18-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>7.2796696998486426E-2</v>
+        <f>Parameters!$C$9*(D18/Parameters!$C$8)/TAN((C18+Parameters!$C$7)*PI()/180)</f>
+        <v>0.0703366630131697</v>
       </c>
       <c r="G18" s="17">
         <f>F18*Parameters!$C$11</f>
-        <v>0.14559339399697285</v>
+        <v>0.1406733260263394</v>
       </c>
       <c r="H18" s="17">
         <f>G18/$G$18</f>
@@ -3554,20 +3559,20 @@
         <v>4</v>
       </c>
       <c r="E19" s="12" t="str">
-        <f t="shared" si="0"/>
+        <f>C19&amp;"° / "&amp;D19&amp;"+"&amp;D19</f>
         <v>70° / 4+4</v>
       </c>
       <c r="F19" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C19*PI()/180)*Parameters!$C$9*(1+(D19-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>5.1297154361627746E-2</v>
+        <f>Parameters!$C$9*(D19/Parameters!$C$8)/TAN((C19+Parameters!$C$7)*PI()/180)</f>
+        <v>0.04689110867544646</v>
       </c>
       <c r="G19" s="20">
         <f>F19*Parameters!$C$11</f>
-        <v>0.10259430872325549</v>
+        <v>0.09378221735089293</v>
       </c>
       <c r="H19" s="20">
         <f>G19/$G$18</f>
-        <v>0.70466321243523322</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -3579,27 +3584,27 @@
       </c>
       <c r="C20" s="15">
         <f>Parameters!C23</f>
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D20" s="15">
         <f>Parameters!G17</f>
         <v>6</v>
       </c>
       <c r="E20" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v>85° / 6+6</v>
+        <f>C20&amp;"° / "&amp;D20&amp;"+"&amp;D20</f>
+        <v>80° / 6+6</v>
       </c>
       <c r="F20" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C20*PI()/180)*Parameters!$C$9*(1+(D20-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>1.7498369728885878E-2</v>
+        <f>Parameters!$C$9*(D20/Parameters!$C$8)/TAN((C20+Parameters!$C$7)*PI()/180)</f>
+        <v>0.022965774175555037</v>
       </c>
       <c r="G20" s="17">
         <f>F20*Parameters!$C$11</f>
-        <v>3.4996739457771757E-2</v>
+        <v>0.045931548351110074</v>
       </c>
       <c r="H20" s="17">
         <f>G20/$G$18</f>
-        <v>0.24037312749573927</v>
+        <v>0.3265121373650463</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -3611,35 +3616,37 @@
       </c>
       <c r="C21" s="18">
         <f>Parameters!C23</f>
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D21" s="18">
         <f>Parameters!G16</f>
         <v>4</v>
       </c>
       <c r="E21" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>85° / 4+4</v>
+        <f>C21&amp;"° / "&amp;D21&amp;"+"&amp;D21</f>
+        <v>80° / 4+4</v>
       </c>
       <c r="F21" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C21*PI()/180)*Parameters!$C$9*(1+(D21-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>1.2330457425536163E-2</v>
+        <f>Parameters!$C$9*(D21/Parameters!$C$8)/TAN((C21+Parameters!$C$7)*PI()/180)</f>
+        <v>0.015310516117036693</v>
       </c>
       <c r="G21" s="20">
         <f>F21*Parameters!$C$11</f>
-        <v>2.4660914851072326E-2</v>
+        <v>0.030621032234073385</v>
       </c>
       <c r="H21" s="20">
         <f>G21/$G$18</f>
-        <v>0.16938210020425151</v>
+        <v>0.21767475824336424</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
     </row>
     <row r="22" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
-      <c r="B22" s="6" t="s">
-        <v>27</v>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Check 1</t>
+        </is>
       </c>
       <c r="C22" s="15">
         <f>Parameters!G8</f>
@@ -3650,16 +3657,16 @@
         <v>4</v>
       </c>
       <c r="E22" s="11" t="str">
-        <f t="shared" si="0"/>
+        <f>C22&amp;"° / "&amp;D22&amp;"+"&amp;D22</f>
         <v>40° / 4+4</v>
       </c>
       <c r="F22" s="16">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C22*PI()/180)*Parameters!$C$9*(1+(D22-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.16796309765159925</v>
+        <f>Parameters!$C$9*(D22/Parameters!$C$8)/TAN((C22+Parameters!$C$7)*PI()/180)</f>
+        <v>0.17500000000000002</v>
       </c>
       <c r="G22" s="17">
         <f>F22*Parameters!$C$11</f>
-        <v>0.3359261953031985</v>
+        <v>0.35000000000000003</v>
       </c>
       <c r="H22" s="17"/>
       <c r="I22" s="2"/>
@@ -3667,8 +3674,10 @@
     </row>
     <row r="23" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
-      <c r="B23" s="9" t="s">
-        <v>28</v>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Check 2</t>
+        </is>
       </c>
       <c r="C23" s="18">
         <f>Parameters!G9</f>
@@ -3679,16 +3688,16 @@
         <v>8</v>
       </c>
       <c r="E23" s="12" t="str">
-        <f t="shared" si="0"/>
+        <f>C23&amp;"° / "&amp;D23&amp;"+"&amp;D23</f>
         <v>35° / 8+8</v>
       </c>
       <c r="F23" s="19">
-        <f>TAN(Parameters!$C$7*PI()/180)/TAN(C23*PI()/180)*Parameters!$C$9*(1+(D23-Parameters!$C$8)*Parameters!$C$10)</f>
-        <v>0.37</v>
+        <f>Parameters!$C$9*(D23/Parameters!$C$8)/TAN((C23+Parameters!$C$7)*PI()/180)</f>
+        <v>0.4171137574079735</v>
       </c>
       <c r="G23" s="20">
         <f>F23*Parameters!$C$11</f>
-        <v>0.74</v>
+        <v>0.834227514815947</v>
       </c>
       <c r="H23" s="20"/>
       <c r="I23" s="2"/>

</xml_diff>